<commit_message>
PBC : harmonisation du format des items ajoutés (couleurs de priorité et de statut, impression, hauteurs, onglets annexes)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QrZoDwZJKb9thfUp96Ro9x
</commit_message>
<xml_diff>
--- a/FPPN_PBC_complete_pointee_20261019.xlsx
+++ b/FPPN_PBC_complete_pointee_20261019.xlsx
@@ -17,8 +17,12 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'PBC Actuariat FPPN'!$B$12:$P$12</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'PBC Actuariat FPPN'!$1:$9</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'PBC Actuariat FPPN'!$A$1:$N$71</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'PBC Actuariat FPPN'!$A$1:$N$136</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Synthèse du pointage'!$5:$5</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Synthèse du pointage'!$A$1:$D$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Détail par mois'!$B$5:$E$1605</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="5">'Points à clarifier'!$5:$5</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="5">'Points à clarifier'!$A$1:$E$42</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
 </workbook>
@@ -281,7 +285,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="96">
+  <cellXfs count="97">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -567,6 +571,9 @@
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -1073,7 +1080,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="61.5" customHeight="1" s="48">
+    <row r="12" ht="72" customHeight="1" s="48">
       <c r="B12" s="70">
         <f>+B11+1</f>
         <v/>
@@ -1107,7 +1114,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="117.75" customHeight="1" s="48">
+    <row r="13" ht="132" customHeight="1" s="48">
       <c r="B13" s="70">
         <f>+B12+1</f>
         <v/>
@@ -1143,7 +1150,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="132" customHeight="1" s="48">
+    <row r="14" ht="147" customHeight="1" s="48">
       <c r="B14" s="70">
         <f>+B13+1</f>
         <v/>
@@ -1179,7 +1186,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="48" customHeight="1" s="48">
+    <row r="15" ht="57" customHeight="1" s="48">
       <c r="B15" s="70">
         <f>+B14+1</f>
         <v/>
@@ -1223,7 +1230,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="117.75" customHeight="1" s="48">
+    <row r="18" ht="132" customHeight="1" s="48">
       <c r="B18" s="70">
         <f>+B15+1</f>
         <v/>
@@ -1259,7 +1266,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="33.75" customHeight="1" s="48">
+    <row r="19" ht="42" customHeight="1" s="48">
       <c r="B19" s="70">
         <f>+B18+1</f>
         <v/>
@@ -1293,7 +1300,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="33.75" customHeight="1" s="48">
+    <row r="20" ht="42" customHeight="1" s="48">
       <c r="B20" s="70">
         <f>+B19+1</f>
         <v/>
@@ -1377,7 +1384,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="33.75" customHeight="1" s="48">
+    <row r="24" ht="42" customHeight="1" s="48">
       <c r="B24" s="70">
         <f>+B23+1</f>
         <v/>
@@ -1453,7 +1460,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="159.75" customHeight="1" s="48">
+    <row r="26" ht="162" customHeight="1" s="48">
       <c r="B26" s="70">
         <f>+B25+1</f>
         <v/>
@@ -1503,7 +1510,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="61.5" customHeight="1" s="48">
+    <row r="29" ht="72" customHeight="1" s="48">
       <c r="B29" s="70">
         <f>+B26+1</f>
         <v/>
@@ -1541,7 +1548,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="75.75" customHeight="1" s="48">
+    <row r="30" ht="87" customHeight="1" s="48">
       <c r="B30" s="70">
         <f>+B29+1</f>
         <v/>
@@ -1579,7 +1586,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="33.75" customHeight="1" s="48">
+    <row r="31" ht="42" customHeight="1" s="48">
       <c r="B31" s="70">
         <f>+B30+1</f>
         <v/>
@@ -1627,7 +1634,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="48" customHeight="1" s="48">
+    <row r="34" ht="57" customHeight="1" s="48">
       <c r="B34" s="70">
         <f>+B31+1</f>
         <v/>
@@ -1661,7 +1668,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="103.5" customHeight="1" s="48">
+    <row r="35" ht="117" customHeight="1" s="48">
       <c r="B35" s="70">
         <f>+B34+1</f>
         <v/>
@@ -1783,7 +1790,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="33.75" customHeight="1" s="48">
+    <row r="40" ht="42" customHeight="1" s="48">
       <c r="B40" s="70">
         <f>+B37+1</f>
         <v/>
@@ -1821,7 +1828,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="117.75" customHeight="1" s="48">
+    <row r="41" ht="132" customHeight="1" s="48">
       <c r="B41" s="70">
         <f>+B40+1</f>
         <v/>
@@ -1861,7 +1868,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="33.75" customHeight="1" s="48">
+    <row r="42" ht="42" customHeight="1" s="48">
       <c r="B42" s="70">
         <f>+B41+1</f>
         <v/>
@@ -1895,7 +1902,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="48" customHeight="1" s="48">
+    <row r="43" ht="57" customHeight="1" s="48">
       <c r="B43" s="70">
         <f>+B42+1</f>
         <v/>
@@ -1973,7 +1980,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="33.75" customHeight="1" s="48">
+    <row r="47" ht="42" customHeight="1" s="48">
       <c r="B47" s="70">
         <f>+B44+1</f>
         <v/>
@@ -2007,7 +2014,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="33.75" customHeight="1" s="48">
+    <row r="48" ht="42" customHeight="1" s="48">
       <c r="B48" s="70">
         <f>+B47+1</f>
         <v/>
@@ -2051,7 +2058,7 @@
         </is>
       </c>
     </row>
-    <row r="51" ht="33.75" customHeight="1" s="48">
+    <row r="51" ht="42" customHeight="1" s="48">
       <c r="B51" s="70">
         <f>+B48+1</f>
         <v/>
@@ -2089,7 +2096,7 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="61.5" customHeight="1" s="48">
+    <row r="52" ht="72" customHeight="1" s="48">
       <c r="B52" s="70">
         <f>+B51+1</f>
         <v/>
@@ -2127,7 +2134,7 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="48" customHeight="1" s="48">
+    <row r="53" ht="57" customHeight="1" s="48">
       <c r="B53" s="70">
         <f>+B52+1</f>
         <v/>
@@ -2165,7 +2172,7 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="33.75" customFormat="1" customHeight="1" s="68">
+    <row r="54" ht="42" customFormat="1" customHeight="1" s="68">
       <c r="B54" s="70">
         <f>+B53+1</f>
         <v/>
@@ -2199,7 +2206,7 @@
         </is>
       </c>
     </row>
-    <row r="55" ht="33.75" customHeight="1" s="48">
+    <row r="55" ht="42" customHeight="1" s="48">
       <c r="B55" s="70">
         <f>+B54+1</f>
         <v/>
@@ -2237,7 +2244,7 @@
         </is>
       </c>
     </row>
-    <row r="56" ht="33.75" customHeight="1" s="48">
+    <row r="56" ht="42" customHeight="1" s="48">
       <c r="B56" s="70">
         <f>+B55+1</f>
         <v/>
@@ -2271,7 +2278,7 @@
         </is>
       </c>
     </row>
-    <row r="57" ht="33.75" customHeight="1" s="48">
+    <row r="57" ht="42" customHeight="1" s="48">
       <c r="B57" s="70">
         <f>+B56+1</f>
         <v/>
@@ -2305,7 +2312,7 @@
         </is>
       </c>
     </row>
-    <row r="58" ht="33.75" customHeight="1" s="48">
+    <row r="58" ht="42" customHeight="1" s="48">
       <c r="B58" s="70">
         <f>+B57+1</f>
         <v/>
@@ -2373,7 +2380,7 @@
         </is>
       </c>
     </row>
-    <row r="60" ht="33.75" customHeight="1" s="48">
+    <row r="60" ht="42" customHeight="1" s="48">
       <c r="B60" s="70">
         <f>+B59+1</f>
         <v/>
@@ -2481,7 +2488,7 @@
         </is>
       </c>
     </row>
-    <row r="63" ht="33.75" customHeight="1" s="48">
+    <row r="63" ht="42" customHeight="1" s="48">
       <c r="B63" s="70">
         <f>+B62+1</f>
         <v/>
@@ -2525,7 +2532,7 @@
         </is>
       </c>
     </row>
-    <row r="66" ht="61.5" customHeight="1" s="48">
+    <row r="66" ht="72" customHeight="1" s="48">
       <c r="B66" s="70">
         <f>+B63+1</f>
         <v/>
@@ -2563,7 +2570,7 @@
         </is>
       </c>
     </row>
-    <row r="67" ht="33.75" customHeight="1" s="48">
+    <row r="67" ht="42" customHeight="1" s="48">
       <c r="B67" s="70">
         <f>+B66+1</f>
         <v/>
@@ -2637,7 +2644,7 @@
         </is>
       </c>
     </row>
-    <row r="69" ht="33.75" customHeight="1" s="48">
+    <row r="69" ht="42" customHeight="1" s="48">
       <c r="B69" s="70">
         <f>+B68+1</f>
         <v/>
@@ -2685,7 +2692,7 @@
         </is>
       </c>
     </row>
-    <row r="72" ht="33.75" customHeight="1" s="48">
+    <row r="72" ht="42" customHeight="1" s="48">
       <c r="B72" s="70">
         <f>+B69+1</f>
         <v/>
@@ -2719,7 +2726,7 @@
         </is>
       </c>
     </row>
-    <row r="73" ht="33.75" customHeight="1" s="48">
+    <row r="73" ht="42" customHeight="1" s="48">
       <c r="B73" s="70">
         <f>+B72+1</f>
         <v/>
@@ -2753,7 +2760,7 @@
         </is>
       </c>
     </row>
-    <row r="74" ht="33.75" customHeight="1" s="48">
+    <row r="74" ht="42" customHeight="1" s="48">
       <c r="B74" s="70">
         <f>+B73+1</f>
         <v/>
@@ -2787,7 +2794,7 @@
         </is>
       </c>
     </row>
-    <row r="75" ht="33.75" customHeight="1" s="48">
+    <row r="75" ht="42" customHeight="1" s="48">
       <c r="B75" s="70">
         <f>+B74+1</f>
         <v/>
@@ -2821,7 +2828,7 @@
         </is>
       </c>
     </row>
-    <row r="76" ht="33.75" customHeight="1" s="48">
+    <row r="76" ht="42" customHeight="1" s="48">
       <c r="B76" s="70">
         <f>+B75+1</f>
         <v/>
@@ -2855,7 +2862,7 @@
         </is>
       </c>
     </row>
-    <row r="77" ht="33.75" customHeight="1" s="48">
+    <row r="77" ht="42" customHeight="1" s="48">
       <c r="B77" s="70">
         <f>+B76+1</f>
         <v/>
@@ -2889,7 +2896,7 @@
         </is>
       </c>
     </row>
-    <row r="78" ht="33.75" customHeight="1" s="48">
+    <row r="78" ht="42" customHeight="1" s="48">
       <c r="B78" s="70">
         <f>+B77+1</f>
         <v/>
@@ -2923,7 +2930,7 @@
         </is>
       </c>
     </row>
-    <row r="79" ht="33.75" customHeight="1" s="48">
+    <row r="79" ht="42" customHeight="1" s="48">
       <c r="B79" s="70">
         <f>+B78+1</f>
         <v/>
@@ -2957,7 +2964,7 @@
         </is>
       </c>
     </row>
-    <row r="80" ht="33.75" customHeight="1" s="48">
+    <row r="80" ht="42" customHeight="1" s="48">
       <c r="B80" s="70">
         <f>+B79+1</f>
         <v/>
@@ -2991,7 +2998,7 @@
         </is>
       </c>
     </row>
-    <row r="81" ht="33.75" customHeight="1" s="48">
+    <row r="81" ht="42" customHeight="1" s="48">
       <c r="B81" s="70">
         <f>+B80+1</f>
         <v/>
@@ -3025,7 +3032,7 @@
         </is>
       </c>
     </row>
-    <row r="82" ht="33.75" customHeight="1" s="48">
+    <row r="82" ht="42" customHeight="1" s="48">
       <c r="B82" s="70">
         <f>+B81+1</f>
         <v/>
@@ -3059,7 +3066,7 @@
         </is>
       </c>
     </row>
-    <row r="83" ht="33.75" customHeight="1" s="48">
+    <row r="83" ht="42" customHeight="1" s="48">
       <c r="B83" s="70">
         <f>+B82+1</f>
         <v/>
@@ -3103,7 +3110,7 @@
         </is>
       </c>
     </row>
-    <row r="86" ht="36" customHeight="1" s="48">
+    <row r="86" ht="57" customHeight="1" s="48">
       <c r="B86" s="70">
         <f>+B83+1</f>
         <v/>
@@ -3141,7 +3148,7 @@
         </is>
       </c>
     </row>
-    <row r="87" ht="36" customHeight="1" s="48">
+    <row r="87" ht="57" customHeight="1" s="48">
       <c r="B87" s="70">
         <f>+B86+1</f>
         <v/>
@@ -3179,7 +3186,7 @@
         </is>
       </c>
     </row>
-    <row r="88" ht="36" customHeight="1" s="48">
+    <row r="88" ht="57" customHeight="1" s="48">
       <c r="B88" s="70">
         <f>+B87+1</f>
         <v/>
@@ -3213,7 +3220,7 @@
         </is>
       </c>
     </row>
-    <row r="89" ht="36" customHeight="1" s="48">
+    <row r="89" ht="42" customHeight="1" s="48">
       <c r="B89" s="70">
         <f>+B88+1</f>
         <v/>
@@ -3247,7 +3254,7 @@
         </is>
       </c>
     </row>
-    <row r="90" ht="36" customHeight="1" s="48">
+    <row r="90" ht="42" customHeight="1" s="48">
       <c r="B90" s="70">
         <f>+B89+1</f>
         <v/>
@@ -3281,7 +3288,7 @@
         </is>
       </c>
     </row>
-    <row r="91" ht="36" customHeight="1" s="48">
+    <row r="91" ht="72" customHeight="1" s="48">
       <c r="B91" s="70">
         <f>+B90+1</f>
         <v/>
@@ -3319,7 +3326,7 @@
         </is>
       </c>
     </row>
-    <row r="92" ht="36" customHeight="1" s="48">
+    <row r="92" ht="57" customHeight="1" s="48">
       <c r="B92" s="70">
         <f>+B91+1</f>
         <v/>
@@ -3357,7 +3364,7 @@
         </is>
       </c>
     </row>
-    <row r="93" ht="36" customHeight="1" s="48">
+    <row r="93" ht="57" customHeight="1" s="48">
       <c r="B93" s="70">
         <f>+B92+1</f>
         <v/>
@@ -3395,7 +3402,7 @@
         </is>
       </c>
     </row>
-    <row r="94" ht="21" customHeight="1" s="48">
+    <row r="94" ht="42" customHeight="1" s="48">
       <c r="B94" s="70">
         <f>+B93+1</f>
         <v/>
@@ -3433,7 +3440,7 @@
         </is>
       </c>
     </row>
-    <row r="95" ht="36" customHeight="1" s="48">
+    <row r="95" ht="42" customHeight="1" s="48">
       <c r="B95" s="70">
         <f>+B94+1</f>
         <v/>
@@ -3471,7 +3478,7 @@
         </is>
       </c>
     </row>
-    <row r="96" ht="21" customHeight="1" s="48">
+    <row r="96" ht="42" customHeight="1" s="48">
       <c r="B96" s="70">
         <f>+B95+1</f>
         <v/>
@@ -3509,7 +3516,7 @@
         </is>
       </c>
     </row>
-    <row r="97" ht="36" customHeight="1" s="48">
+    <row r="97" ht="57" customHeight="1" s="48">
       <c r="B97" s="70">
         <f>+B96+1</f>
         <v/>
@@ -3547,7 +3554,7 @@
         </is>
       </c>
     </row>
-    <row r="98" ht="36" customHeight="1" s="48">
+    <row r="98" ht="42" customHeight="1" s="48">
       <c r="B98" s="70">
         <f>+B97+1</f>
         <v/>
@@ -3585,7 +3592,7 @@
         </is>
       </c>
     </row>
-    <row r="99" ht="36" customHeight="1" s="48">
+    <row r="99" ht="42" customHeight="1" s="48">
       <c r="B99" s="70">
         <f>+B98+1</f>
         <v/>
@@ -3619,7 +3626,7 @@
         </is>
       </c>
     </row>
-    <row r="100" ht="36" customHeight="1" s="48">
+    <row r="100" ht="57" customHeight="1" s="48">
       <c r="B100" s="70">
         <f>+B99+1</f>
         <v/>
@@ -3663,7 +3670,7 @@
         </is>
       </c>
     </row>
-    <row r="103" ht="51" customHeight="1" s="48">
+    <row r="103" ht="87" customHeight="1" s="48">
       <c r="B103" s="70">
         <f>+B100+1</f>
         <v/>
@@ -3701,7 +3708,7 @@
         </is>
       </c>
     </row>
-    <row r="104" ht="36" customHeight="1" s="48">
+    <row r="104" ht="57" customHeight="1" s="48">
       <c r="B104" s="70">
         <f>+B103+1</f>
         <v/>
@@ -3735,7 +3742,7 @@
         </is>
       </c>
     </row>
-    <row r="105" ht="36" customHeight="1" s="48">
+    <row r="105" ht="42" customHeight="1" s="48">
       <c r="B105" s="70">
         <f>+B104+1</f>
         <v/>
@@ -3773,7 +3780,7 @@
         </is>
       </c>
     </row>
-    <row r="106" ht="36" customHeight="1" s="48">
+    <row r="106" ht="42" customHeight="1" s="48">
       <c r="B106" s="70">
         <f>+B105+1</f>
         <v/>
@@ -3807,7 +3814,7 @@
         </is>
       </c>
     </row>
-    <row r="107" ht="36" customHeight="1" s="48">
+    <row r="107" ht="42" customHeight="1" s="48">
       <c r="B107" s="70">
         <f>+B106+1</f>
         <v/>
@@ -3845,7 +3852,7 @@
         </is>
       </c>
     </row>
-    <row r="108" ht="36" customHeight="1" s="48">
+    <row r="108" ht="42" customHeight="1" s="48">
       <c r="B108" s="70">
         <f>+B107+1</f>
         <v/>
@@ -3883,7 +3890,7 @@
         </is>
       </c>
     </row>
-    <row r="109" ht="36" customHeight="1" s="48">
+    <row r="109" ht="42" customHeight="1" s="48">
       <c r="B109" s="70">
         <f>+B108+1</f>
         <v/>
@@ -3917,7 +3924,7 @@
         </is>
       </c>
     </row>
-    <row r="110" ht="36" customHeight="1" s="48">
+    <row r="110" ht="42" customHeight="1" s="48">
       <c r="B110" s="70">
         <f>+B109+1</f>
         <v/>
@@ -3951,7 +3958,7 @@
         </is>
       </c>
     </row>
-    <row r="111" ht="36" customHeight="1" s="48">
+    <row r="111" ht="42" customHeight="1" s="48">
       <c r="B111" s="70">
         <f>+B110+1</f>
         <v/>
@@ -3995,7 +4002,7 @@
         </is>
       </c>
     </row>
-    <row r="114" ht="21" customHeight="1" s="48">
+    <row r="114" ht="42" customHeight="1" s="48">
       <c r="B114" s="70">
         <f>+B111+1</f>
         <v/>
@@ -4033,7 +4040,7 @@
         </is>
       </c>
     </row>
-    <row r="115" ht="36" customHeight="1" s="48">
+    <row r="115" ht="42" customHeight="1" s="48">
       <c r="B115" s="70">
         <f>+B114+1</f>
         <v/>
@@ -4071,7 +4078,7 @@
         </is>
       </c>
     </row>
-    <row r="116" ht="36" customHeight="1" s="48">
+    <row r="116" ht="42" customHeight="1" s="48">
       <c r="B116" s="70">
         <f>+B115+1</f>
         <v/>
@@ -4109,7 +4116,7 @@
         </is>
       </c>
     </row>
-    <row r="117" ht="21" customHeight="1" s="48">
+    <row r="117" ht="42" customHeight="1" s="48">
       <c r="B117" s="70">
         <f>+B116+1</f>
         <v/>
@@ -4143,7 +4150,7 @@
         </is>
       </c>
     </row>
-    <row r="118" ht="36" customHeight="1" s="48">
+    <row r="118" ht="42" customHeight="1" s="48">
       <c r="B118" s="70">
         <f>+B117+1</f>
         <v/>
@@ -4177,7 +4184,7 @@
         </is>
       </c>
     </row>
-    <row r="119" ht="21" customHeight="1" s="48">
+    <row r="119" ht="42" customHeight="1" s="48">
       <c r="B119" s="70">
         <f>+B118+1</f>
         <v/>
@@ -4211,7 +4218,7 @@
         </is>
       </c>
     </row>
-    <row r="120" ht="21" customHeight="1" s="48">
+    <row r="120" ht="42" customHeight="1" s="48">
       <c r="B120" s="70">
         <f>+B119+1</f>
         <v/>
@@ -4245,7 +4252,7 @@
         </is>
       </c>
     </row>
-    <row r="121" ht="36" customHeight="1" s="48">
+    <row r="121" ht="42" customHeight="1" s="48">
       <c r="B121" s="70">
         <f>+B120+1</f>
         <v/>
@@ -4279,7 +4286,7 @@
         </is>
       </c>
     </row>
-    <row r="122" ht="21" customHeight="1" s="48">
+    <row r="122" ht="42" customHeight="1" s="48">
       <c r="B122" s="70">
         <f>+B121+1</f>
         <v/>
@@ -4317,7 +4324,7 @@
         </is>
       </c>
     </row>
-    <row r="123" ht="21" customHeight="1" s="48">
+    <row r="123" ht="42" customHeight="1" s="48">
       <c r="B123" s="70">
         <f>+B122+1</f>
         <v/>
@@ -4351,7 +4358,7 @@
         </is>
       </c>
     </row>
-    <row r="124" ht="21" customHeight="1" s="48">
+    <row r="124" ht="42" customHeight="1" s="48">
       <c r="B124" s="70">
         <f>+B123+1</f>
         <v/>
@@ -4389,7 +4396,7 @@
         </is>
       </c>
     </row>
-    <row r="125" ht="21" customHeight="1" s="48">
+    <row r="125" ht="42" customHeight="1" s="48">
       <c r="B125" s="70">
         <f>+B124+1</f>
         <v/>
@@ -4437,7 +4444,7 @@
         </is>
       </c>
     </row>
-    <row r="128" ht="36" customHeight="1" s="48">
+    <row r="128" ht="42" customHeight="1" s="48">
       <c r="B128" s="70">
         <f>+B125+1</f>
         <v/>
@@ -4475,7 +4482,7 @@
         </is>
       </c>
     </row>
-    <row r="129" ht="21" customHeight="1" s="48">
+    <row r="129" ht="42" customHeight="1" s="48">
       <c r="B129" s="70">
         <f>+B128+1</f>
         <v/>
@@ -4509,7 +4516,7 @@
         </is>
       </c>
     </row>
-    <row r="130" ht="21" customHeight="1" s="48">
+    <row r="130" ht="42" customHeight="1" s="48">
       <c r="B130" s="70">
         <f>+B129+1</f>
         <v/>
@@ -4543,7 +4550,7 @@
         </is>
       </c>
     </row>
-    <row r="131" ht="21" customHeight="1" s="48">
+    <row r="131" ht="42" customHeight="1" s="48">
       <c r="B131" s="70">
         <f>+B130+1</f>
         <v/>
@@ -4577,7 +4584,7 @@
         </is>
       </c>
     </row>
-    <row r="132" ht="21" customHeight="1" s="48">
+    <row r="132" ht="42" customHeight="1" s="48">
       <c r="B132" s="70">
         <f>+B131+1</f>
         <v/>
@@ -4611,7 +4618,7 @@
         </is>
       </c>
     </row>
-    <row r="133" ht="21" customHeight="1" s="48">
+    <row r="133" ht="42" customHeight="1" s="48">
       <c r="B133" s="70">
         <f>+B132+1</f>
         <v/>
@@ -4649,7 +4656,7 @@
         </is>
       </c>
     </row>
-    <row r="134" ht="21" customHeight="1" s="48">
+    <row r="134" ht="42" customHeight="1" s="48">
       <c r="B134" s="70">
         <f>+B133+1</f>
         <v/>
@@ -4687,7 +4694,7 @@
         </is>
       </c>
     </row>
-    <row r="135" ht="21" customHeight="1" s="48">
+    <row r="135" ht="42" customHeight="1" s="48">
       <c r="B135" s="70">
         <f>+B134+1</f>
         <v/>
@@ -4728,7 +4735,7 @@
     <mergeCell ref="C5:M5"/>
     <mergeCell ref="C4:M4"/>
   </mergeCells>
-  <conditionalFormatting sqref="M11:M69">
+  <conditionalFormatting sqref="M11:M135">
     <cfRule type="cellIs" rank="0" priority="2" equalAverage="0" operator="equal" aboveAverage="0" dxfId="6" text="" percent="0" bottom="0">
       <formula>"Partiellement Reçu"</formula>
     </cfRule>
@@ -4739,7 +4746,7 @@
       <formula>"Reçu"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E11:E69">
+  <conditionalFormatting sqref="E11:E135">
     <cfRule type="cellIs" rank="0" priority="5" equalAverage="0" operator="equal" aboveAverage="0" dxfId="9" text="" percent="0" bottom="0">
       <formula>"Faible"</formula>
     </cfRule>
@@ -4782,7 +4789,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B2:D9"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
@@ -4852,7 +4859,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="60" customHeight="1" s="48">
+    <row r="8" ht="87" customHeight="1" s="48">
       <c r="B8" s="94" t="inlineStr">
         <is>
           <t>Non Reçu</t>
@@ -4868,7 +4875,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="18" customHeight="1" s="48">
+    <row r="9" ht="30" customHeight="1" s="48">
       <c r="B9" s="94" t="inlineStr">
         <is>
           <t>Total</t>
@@ -4887,7 +4894,7 @@
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup orientation="landscape" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
 </worksheet>
 </file>
 
@@ -42148,7 +42155,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B2:E42"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
@@ -42195,8 +42202,8 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="60" customHeight="1" s="48">
-      <c r="B6" s="94" t="n">
+    <row r="6" ht="72" customHeight="1" s="48">
+      <c r="B6" s="96" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="95" t="inlineStr">
@@ -42215,8 +42222,8 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="31.5" customHeight="1" s="48">
-      <c r="B7" s="94" t="n">
+    <row r="7" ht="42" customHeight="1" s="48">
+      <c r="B7" s="96" t="n">
         <v>2</v>
       </c>
       <c r="C7" s="95" t="inlineStr">
@@ -42235,8 +42242,8 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="45.75" customHeight="1" s="48">
-      <c r="B8" s="94" t="n">
+    <row r="8" ht="57" customHeight="1" s="48">
+      <c r="B8" s="96" t="n">
         <v>3</v>
       </c>
       <c r="C8" s="95" t="inlineStr">
@@ -42255,8 +42262,8 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="31.5" customHeight="1" s="48">
-      <c r="B9" s="94" t="n">
+    <row r="9" ht="42" customHeight="1" s="48">
+      <c r="B9" s="96" t="n">
         <v>4</v>
       </c>
       <c r="C9" s="95" t="inlineStr">
@@ -42275,8 +42282,8 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="45.75" customHeight="1" s="48">
-      <c r="B10" s="94" t="n">
+    <row r="10" ht="57" customHeight="1" s="48">
+      <c r="B10" s="96" t="n">
         <v>5</v>
       </c>
       <c r="C10" s="95" t="inlineStr">
@@ -42295,8 +42302,8 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="31.5" customHeight="1" s="48">
-      <c r="B11" s="94" t="n">
+    <row r="11" ht="42" customHeight="1" s="48">
+      <c r="B11" s="96" t="n">
         <v>6</v>
       </c>
       <c r="C11" s="95" t="inlineStr">
@@ -42315,8 +42322,8 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="31.5" customHeight="1" s="48">
-      <c r="B12" s="94" t="n">
+    <row r="12" ht="42" customHeight="1" s="48">
+      <c r="B12" s="96" t="n">
         <v>7</v>
       </c>
       <c r="C12" s="95" t="inlineStr">
@@ -42335,8 +42342,8 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="45.75" customHeight="1" s="48">
-      <c r="B13" s="94" t="n">
+    <row r="13" ht="72" customHeight="1" s="48">
+      <c r="B13" s="96" t="n">
         <v>8</v>
       </c>
       <c r="C13" s="95" t="inlineStr">
@@ -42355,8 +42362,8 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="31.5" customHeight="1" s="48">
-      <c r="B14" s="94" t="n">
+    <row r="14" ht="42" customHeight="1" s="48">
+      <c r="B14" s="96" t="n">
         <v>9</v>
       </c>
       <c r="C14" s="95" t="inlineStr">
@@ -42375,8 +42382,8 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="31.5" customHeight="1" s="48">
-      <c r="B15" s="94" t="n">
+    <row r="15" ht="57" customHeight="1" s="48">
+      <c r="B15" s="96" t="n">
         <v>10</v>
       </c>
       <c r="C15" s="95" t="inlineStr">
@@ -42395,8 +42402,8 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="60" customHeight="1" s="48">
-      <c r="B16" s="94" t="n">
+    <row r="16" ht="87" customHeight="1" s="48">
+      <c r="B16" s="96" t="n">
         <v>11</v>
       </c>
       <c r="C16" s="95" t="inlineStr">
@@ -42415,8 +42422,8 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="73.5" customHeight="1" s="48">
-      <c r="B17" s="94" t="n">
+    <row r="17" ht="102" customHeight="1" s="48">
+      <c r="B17" s="96" t="n">
         <v>12</v>
       </c>
       <c r="C17" s="95" t="inlineStr">
@@ -42435,8 +42442,8 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="45.75" customHeight="1" s="48">
-      <c r="B18" s="94" t="n">
+    <row r="18" ht="57" customHeight="1" s="48">
+      <c r="B18" s="96" t="n">
         <v>13</v>
       </c>
       <c r="C18" s="95" t="inlineStr">
@@ -42455,8 +42462,8 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="31.5" customHeight="1" s="48">
-      <c r="B19" s="94" t="n">
+    <row r="19" ht="42" customHeight="1" s="48">
+      <c r="B19" s="96" t="n">
         <v>14</v>
       </c>
       <c r="C19" s="95" t="inlineStr">
@@ -42475,8 +42482,8 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="60" customHeight="1" s="48">
-      <c r="B20" s="94" t="n">
+    <row r="20" ht="87" customHeight="1" s="48">
+      <c r="B20" s="96" t="n">
         <v>15</v>
       </c>
       <c r="C20" s="95" t="inlineStr">
@@ -42495,8 +42502,8 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="60" customHeight="1" s="48">
-      <c r="B21" s="94" t="n">
+    <row r="21" ht="72" customHeight="1" s="48">
+      <c r="B21" s="96" t="n">
         <v>16</v>
       </c>
       <c r="C21" s="95" t="inlineStr">
@@ -42515,8 +42522,8 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="31.5" customHeight="1" s="48">
-      <c r="B22" s="94" t="n">
+    <row r="22" ht="57" customHeight="1" s="48">
+      <c r="B22" s="96" t="n">
         <v>17</v>
       </c>
       <c r="C22" s="95" t="inlineStr">
@@ -42535,8 +42542,8 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="45.75" customHeight="1" s="48">
-      <c r="B23" s="94" t="n">
+    <row r="23" ht="57" customHeight="1" s="48">
+      <c r="B23" s="96" t="n">
         <v>18</v>
       </c>
       <c r="C23" s="95" t="inlineStr">
@@ -42555,8 +42562,8 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="18" customHeight="1" s="48">
-      <c r="B24" s="94" t="n">
+    <row r="24" ht="42" customHeight="1" s="48">
+      <c r="B24" s="96" t="n">
         <v>19</v>
       </c>
       <c r="C24" s="95" t="inlineStr">
@@ -42575,8 +42582,8 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="31.5" customHeight="1" s="48">
-      <c r="B25" s="94" t="n">
+    <row r="25" ht="57" customHeight="1" s="48">
+      <c r="B25" s="96" t="n">
         <v>20</v>
       </c>
       <c r="C25" s="95" t="inlineStr">
@@ -42595,8 +42602,8 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="31.5" customHeight="1" s="48">
-      <c r="B26" s="94" t="n">
+    <row r="26" ht="42" customHeight="1" s="48">
+      <c r="B26" s="96" t="n">
         <v>21</v>
       </c>
       <c r="C26" s="95" t="inlineStr">
@@ -42615,11 +42622,9 @@
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="B27" s="94" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
+    <row r="27" ht="42" customHeight="1" s="48">
+      <c r="B27" s="96" t="n">
+        <v>22</v>
       </c>
       <c r="C27" s="95" t="inlineStr">
         <is>
@@ -42637,11 +42642,9 @@
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="B28" s="94" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
+    <row r="28" ht="42" customHeight="1" s="48">
+      <c r="B28" s="96" t="n">
+        <v>23</v>
       </c>
       <c r="C28" s="95" t="inlineStr">
         <is>
@@ -42659,11 +42662,9 @@
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="B29" s="94" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
+    <row r="29" ht="42" customHeight="1" s="48">
+      <c r="B29" s="96" t="n">
+        <v>24</v>
       </c>
       <c r="C29" s="95" t="inlineStr">
         <is>
@@ -42681,11 +42682,9 @@
         </is>
       </c>
     </row>
-    <row r="30" s="48">
-      <c r="B30" s="94" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
+    <row r="30" ht="42" customHeight="1" s="48">
+      <c r="B30" s="96" t="n">
+        <v>25</v>
       </c>
       <c r="C30" s="95" t="inlineStr">
         <is>
@@ -42703,11 +42702,9 @@
         </is>
       </c>
     </row>
-    <row r="31" s="48">
-      <c r="B31" s="94" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
+    <row r="31" ht="87" customHeight="1" s="48">
+      <c r="B31" s="96" t="n">
+        <v>26</v>
       </c>
       <c r="C31" s="95" t="inlineStr">
         <is>
@@ -42725,11 +42722,9 @@
         </is>
       </c>
     </row>
-    <row r="32" s="48">
-      <c r="B32" s="94" t="inlineStr">
-        <is>
-          <t>27</t>
-        </is>
+    <row r="32" ht="72" customHeight="1" s="48">
+      <c r="B32" s="96" t="n">
+        <v>27</v>
       </c>
       <c r="C32" s="95" t="inlineStr">
         <is>
@@ -42747,11 +42742,9 @@
         </is>
       </c>
     </row>
-    <row r="33" s="48">
-      <c r="B33" s="94" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
+    <row r="33" ht="72" customHeight="1" s="48">
+      <c r="B33" s="96" t="n">
+        <v>28</v>
       </c>
       <c r="C33" s="95" t="inlineStr">
         <is>
@@ -42769,11 +42762,9 @@
         </is>
       </c>
     </row>
-    <row r="34" s="48">
-      <c r="B34" s="94" t="inlineStr">
-        <is>
-          <t>29</t>
-        </is>
+    <row r="34" ht="57" customHeight="1" s="48">
+      <c r="B34" s="96" t="n">
+        <v>29</v>
       </c>
       <c r="C34" s="95" t="inlineStr">
         <is>
@@ -42791,8 +42782,8 @@
         </is>
       </c>
     </row>
-    <row r="35" s="48">
-      <c r="B35" s="94" t="n">
+    <row r="35" ht="57" customHeight="1" s="48">
+      <c r="B35" s="96" t="n">
         <v>30</v>
       </c>
       <c r="C35" s="95" t="inlineStr">
@@ -42811,8 +42802,8 @@
         </is>
       </c>
     </row>
-    <row r="36" s="48">
-      <c r="B36" s="94" t="n">
+    <row r="36" ht="57" customHeight="1" s="48">
+      <c r="B36" s="96" t="n">
         <v>31</v>
       </c>
       <c r="C36" s="95" t="inlineStr">
@@ -42831,8 +42822,8 @@
         </is>
       </c>
     </row>
-    <row r="37" s="48">
-      <c r="B37" s="94" t="n">
+    <row r="37" ht="42" customHeight="1" s="48">
+      <c r="B37" s="96" t="n">
         <v>32</v>
       </c>
       <c r="C37" s="95" t="inlineStr">
@@ -42851,8 +42842,8 @@
         </is>
       </c>
     </row>
-    <row r="38" s="48">
-      <c r="B38" s="94" t="n">
+    <row r="38" ht="57" customHeight="1" s="48">
+      <c r="B38" s="96" t="n">
         <v>33</v>
       </c>
       <c r="C38" s="95" t="inlineStr">
@@ -42871,8 +42862,8 @@
         </is>
       </c>
     </row>
-    <row r="39" s="48">
-      <c r="B39" s="94" t="n">
+    <row r="39" ht="42" customHeight="1" s="48">
+      <c r="B39" s="96" t="n">
         <v>34</v>
       </c>
       <c r="C39" s="95" t="inlineStr">
@@ -42891,8 +42882,8 @@
         </is>
       </c>
     </row>
-    <row r="40" s="48">
-      <c r="B40" s="94" t="n">
+    <row r="40" ht="57" customHeight="1" s="48">
+      <c r="B40" s="96" t="n">
         <v>35</v>
       </c>
       <c r="C40" s="95" t="inlineStr">
@@ -42911,8 +42902,8 @@
         </is>
       </c>
     </row>
-    <row r="41" s="48">
-      <c r="B41" s="94" t="n">
+    <row r="41" ht="42" customHeight="1" s="48">
+      <c r="B41" s="96" t="n">
         <v>36</v>
       </c>
       <c r="C41" s="95" t="inlineStr">
@@ -42931,8 +42922,8 @@
         </is>
       </c>
     </row>
-    <row r="42" s="48">
-      <c r="B42" s="94" t="n">
+    <row r="42" ht="31.5" customHeight="1" s="48">
+      <c r="B42" s="96" t="n">
         <v>37</v>
       </c>
       <c r="C42" s="95" t="inlineStr">
@@ -42954,6 +42945,6 @@
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup orientation="landscape" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
 </worksheet>
 </file>
</xml_diff>